<commit_message>
final commit to make sure everything is updated in github
</commit_message>
<xml_diff>
--- a/data/bike-rides.xlsx
+++ b/data/bike-rides.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="12">
   <si>
     <t>Date</t>
   </si>
@@ -495,7 +495,7 @@
         <v>394.0</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E6" s="6">
         <v>68.0</v>
@@ -547,7 +547,7 @@
         <v>325.0</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E8" s="6">
         <v>72.0</v>
@@ -625,7 +625,7 @@
         <v>330.0</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E11" s="6">
         <v>65.0</v>
@@ -677,7 +677,7 @@
         <v>381.0</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E13" s="6">
         <v>70.0</v>
@@ -794,6 +794,58 @@
       </c>
       <c r="H17" s="6">
         <v>5.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7">
+        <v>46168.0</v>
+      </c>
+      <c r="B18" s="5">
+        <v>0.5138888888888888</v>
+      </c>
+      <c r="C18" s="6">
+        <v>300.0</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="6">
+        <v>65.0</v>
+      </c>
+      <c r="F18" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H18" s="6">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7">
+        <v>46168.0</v>
+      </c>
+      <c r="B19" s="5">
+        <v>0.2604166666666667</v>
+      </c>
+      <c r="C19" s="6">
+        <v>310.0</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19" s="6">
+        <v>66.0</v>
+      </c>
+      <c r="F19" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H19" s="6">
+        <v>4.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>